<commit_message>
auto: 2026-07-14 05:33 (11件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R8f1582891d774265"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R0931ace479eb467d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Rd071f073c8ff4536"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R5d346cde1a1d46a5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rfff8cf8c3bd14591"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="R2c7a35db017a4c59"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -200,7 +200,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -211,7 +211,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -222,7 +222,7 @@
         <x:color rgb="FF7A4D00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -233,7 +233,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F3EA"/>
         </x:patternFill>
       </x:fill>
@@ -244,7 +244,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -255,7 +255,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -266,7 +266,7 @@
         <x:color rgb="FF7A4D00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -277,7 +277,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F3EA"/>
         </x:patternFill>
       </x:fill>
@@ -288,7 +288,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -299,7 +299,7 @@
         <x:color rgb="FFA61B1B"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFCE8E6"/>
         </x:patternFill>
       </x:fill>
@@ -310,7 +310,7 @@
         <x:color rgb="FF7A4D00"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFFFF2CC"/>
         </x:patternFill>
       </x:fill>
@@ -321,7 +321,7 @@
         <x:color rgb="FF216E39"/>
       </x:font>
       <x:fill>
-        <x:patternFill patternType="solid">
+        <x:patternFill>
           <x:bgColor rgb="FFE7F3EA"/>
         </x:patternFill>
       </x:fill>
@@ -1992,7 +1992,7 @@
         <x:v>イタリア</x:v>
       </x:c>
       <x:c r="D33" s="26" t="str">
-        <x:v>除外</x:v>
+        <x:v>営業表示あり</x:v>
       </x:c>
       <x:c r="E33" s="26" t="str">
         <x:v>国内ECのため除外</x:v>
@@ -2022,7 +2022,9 @@
       <x:c r="V33" s="26" t="str">
         <x:v>除外</x:v>
       </x:c>
-      <x:c r="W33" s="26" t="str"/>
+      <x:c r="W33" s="26" t="str">
+        <x:v>現行サイトは営業表示あり。ただし日本向け国内ECのためBUYMA買付候補から除外</x:v>
+      </x:c>
       <x:c r="X33" s="27" t="str"/>
       <x:c r="Y33" s="26" t="str"/>
       <x:c r="Z33" s="26" t="str"/>

</xml_diff>

<commit_message>
auto: 2026-07-14 06:43 (10件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R5d346cde1a1d46a5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rfff8cf8c3bd14591"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="R2c7a35db017a4c59"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R2723a16631424c1e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R1b9740a2d91e4846"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Ra6bfb1e859b34d6e"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
auto: 2026-07-14 07:23 (8件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R2723a16631424c1e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R1b9740a2d91e4846"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Ra6bfb1e859b34d6e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="Ra1af4806ff274f33"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R81a0b49715b143a2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Rbfae003e6aa64226"/>
   </x:sheets>
 </x:workbook>
 </file>

</xml_diff>

<commit_message>
auto: 2026-07-14 08:33 (8件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="Ra1af4806ff274f33"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R81a0b49715b143a2"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Rbfae003e6aa64226"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R8ced6b7210604203"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R7f336433664a40b7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Ra66498ec73e94cfa"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -4458,26 +4458,14 @@
     <x:mergeCell ref="A1:Z1"/>
     <x:mergeCell ref="A2:Z2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="D5:D92">
-    <x:cfRule type="containsText" dxfId="0" priority="1" operator="containsText" text="STOP"/>
-    <x:cfRule type="containsText" dxfId="1" priority="2" operator="containsText" text="除外"/>
-    <x:cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="保留"/>
-    <x:cfRule type="containsText" dxfId="3" priority="4" operator="containsText" text="確認済み"/>
-  </x:conditionalFormatting>
-  <x:conditionalFormatting sqref="V5:V92">
-    <x:cfRule type="containsText" dxfId="4" priority="5" operator="containsText" text="STOP"/>
-    <x:cfRule type="containsText" dxfId="5" priority="6" operator="containsText" text="除外"/>
-    <x:cfRule type="containsText" dxfId="6" priority="7" operator="containsText" text="保留"/>
-    <x:cfRule type="containsText" dxfId="7" priority="8" operator="containsText" text="確認済み"/>
-  </x:conditionalFormatting>
   <x:dataValidations count="3">
-    <x:dataValidation type="list" sqref="D5:D92">
+    <x:dataValidation type="list" sqref="D5:D104">
       <x:formula1>"未確認,営業表示あり,URL・名称・運営変更,要再確認,閉鎖,除外"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="M5:M92">
+    <x:dataValidation type="list" sqref="M5:M104">
       <x:formula1>"未確認,単独販売,提携店型,マーケットプレイス,不明"</x:formula1>
     </x:dataValidation>
-    <x:dataValidation type="list" sqref="V5:V92">
+    <x:dataValidation type="list" sqref="V5:V104">
       <x:formula1>"未確認,使用可候補,保留,除外"</x:formula1>
     </x:dataValidation>
   </x:dataValidations>

</xml_diff>

<commit_message>
auto: 2026-07-14 08:43 (9件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R8ced6b7210604203"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="R7f336433664a40b7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Ra66498ec73e94cfa"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="Rd6a7b1df136341bf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rb24a0073d662470a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="R3ac007bfba944cc7"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -8700,12 +8700,6 @@
     <x:mergeCell ref="A1:R1"/>
     <x:mergeCell ref="A2:R2"/>
   </x:mergeCells>
-  <x:conditionalFormatting sqref="O5:O204">
-    <x:cfRule type="containsText" dxfId="8" priority="1" operator="containsText" text="STOP"/>
-    <x:cfRule type="containsText" dxfId="9" priority="2" operator="containsText" text="除外"/>
-    <x:cfRule type="containsText" dxfId="10" priority="3" operator="containsText" text="保留"/>
-    <x:cfRule type="containsText" dxfId="11" priority="4" operator="containsText" text="確認済み"/>
-  </x:conditionalFormatting>
   <x:dataValidations count="1">
     <x:dataValidation type="list" sqref="O5:O204">
       <x:formula1>"未確認,注文可,保留,除外"</x:formula1>

</xml_diff>

<commit_message>
auto: 2026-07-15 06:24 (7件)
</commit_message>
<xml_diff>
--- a/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
+++ b/01_プロジェクト/BUYMA購入者配布資料/BUYMA_ショップ確認台帳_購入者版.xlsx
@@ -2,9 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="Rd6a7b1df136341bf"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Rb24a0073d662470a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="R3ac007bfba944cc7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="ショップ現況監査" sheetId="1" r:id="R3ea6b0638585478a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="使い方" sheetId="2" r:id="Re8f515f2b32744c5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="注文前確認" sheetId="3" r:id="Ra52c4d6ad7c942d6"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -851,7 +851,7 @@
         <x:v>https://www.saksfifthavenue.com/</x:v>
       </x:c>
       <x:c r="G8" s="26" t="str">
-        <x:v>現行サイト。親会社の再建・名称変更後のため、請求主体と返品条件を注文時に再確認</x:v>
+        <x:v>現行サイト。請求主体、販売元、返品条件を注文時に再確認</x:v>
       </x:c>
       <x:c r="H8" s="26" t="str"/>
       <x:c r="I8" s="26" t="str"/>
@@ -943,7 +943,7 @@
         <x:v>https://www.neimanmarcus.com/</x:v>
       </x:c>
       <x:c r="G10" s="26" t="str">
-        <x:v>現行サイト。親会社の再建後のため、閉店情報とEC継続を分けて確認</x:v>
+        <x:v>現行サイト。販売元、配送条件、返品条件を注文時に再確認</x:v>
       </x:c>
       <x:c r="H10" s="26" t="str"/>
       <x:c r="I10" s="26" t="str"/>
@@ -1173,7 +1173,7 @@
         <x:v>https://shop.trendcincinnati.com/</x:v>
       </x:c>
       <x:c r="G15" s="26" t="str">
-        <x:v>現行サイト。実店舗閉鎖・オンライン運営の表示があるため発送条件を確認</x:v>
+        <x:v>現行サイト。現在の販売主体、発送条件、返品条件を確認</x:v>
       </x:c>
       <x:c r="H15" s="26" t="str"/>
       <x:c r="I15" s="26" t="str"/>
@@ -1210,10 +1210,10 @@
         <x:v>アメリカ</x:v>
       </x:c>
       <x:c r="D16" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E16" s="26" t="str">
-        <x:v>EC終了</x:v>
+        <x:v>現行の海外ECを確認できず</x:v>
       </x:c>
       <x:c r="F16" s="26" t="str">
         <x:v>http://ronherman.com/</x:v>
@@ -1486,10 +1486,10 @@
         <x:v>アラブ首長国連邦</x:v>
       </x:c>
       <x:c r="D22" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E22" s="26" t="str">
-        <x:v>EC終了</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F22" s="26" t="str">
         <x:v>https://www.boutique1.com/</x:v>
@@ -1817,7 +1817,7 @@
         <x:v>https://www.theoutnet.com/en-us/</x:v>
       </x:c>
       <x:c r="G29" s="26" t="str">
-        <x:v>現行サイト。運営移行後の請求主体、返品先、規約を再確認</x:v>
+        <x:v>現行サイト。請求主体、販売元、返品先、規約を再確認</x:v>
       </x:c>
       <x:c r="H29" s="26" t="str"/>
       <x:c r="I29" s="26" t="str"/>
@@ -1900,10 +1900,10 @@
         <x:v>イギリス</x:v>
       </x:c>
       <x:c r="D31" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E31" s="26" t="str">
-        <x:v>EC終了・再始動待ち</x:v>
+        <x:v>公式EC停止・再始動待ち</x:v>
       </x:c>
       <x:c r="F31" s="26" t="str">
         <x:v>https://matchesfashion.com/</x:v>
@@ -1946,10 +1946,10 @@
         <x:v>イタリア</x:v>
       </x:c>
       <x:c r="D32" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E32" s="26" t="str">
-        <x:v>EC終了</x:v>
+        <x:v>公式EC閉鎖</x:v>
       </x:c>
       <x:c r="F32" s="26" t="str">
         <x:v>https://frmoda.com/</x:v>
@@ -2224,10 +2224,10 @@
         <x:v>イタリア</x:v>
       </x:c>
       <x:c r="D38" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E38" s="26" t="str">
-        <x:v>閉鎖扱い</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F38" s="26" t="str"/>
       <x:c r="G38" s="26" t="str">
@@ -2544,10 +2544,10 @@
         <x:v>イタリア</x:v>
       </x:c>
       <x:c r="D45" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E45" s="26" t="str">
-        <x:v>EC終了</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F45" s="26" t="str"/>
       <x:c r="G45" s="26" t="str">
@@ -2818,10 +2818,10 @@
         <x:v>イタリア</x:v>
       </x:c>
       <x:c r="D51" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E51" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F51" s="26" t="str"/>
       <x:c r="G51" s="26" t="str">
@@ -3092,10 +3092,10 @@
         <x:v>オーストラリア</x:v>
       </x:c>
       <x:c r="D57" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E57" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F57" s="26" t="str"/>
       <x:c r="G57" s="26" t="str">
@@ -3228,10 +3228,10 @@
         <x:v>オーストラリア</x:v>
       </x:c>
       <x:c r="D60" s="26" t="str">
-        <x:v>閉鎖</x:v>
+        <x:v>公式EC確認不可・閉鎖告知等</x:v>
       </x:c>
       <x:c r="E60" s="26" t="str">
-        <x:v>閉鎖扱い</x:v>
+        <x:v>現行公式ECを確認できず</x:v>
       </x:c>
       <x:c r="F60" s="26" t="str"/>
       <x:c r="G60" s="26" t="str">
@@ -3281,7 +3281,7 @@
         <x:v>https://www.ssense.com/ja-jp/men/sale</x:v>
       </x:c>
       <x:c r="G61" s="26" t="str">
-        <x:v>現行サイト。再建・運営変更後の規約、決済、返品条件を注文時に確認</x:v>
+        <x:v>現行サイト。販売元、決済、配送、返品条件を注文時に確認</x:v>
       </x:c>
       <x:c r="H61" s="26" t="str"/>
       <x:c r="I61" s="26" t="str"/>
@@ -4460,7 +4460,7 @@
   </x:mergeCells>
   <x:dataValidations count="3">
     <x:dataValidation type="list" sqref="D5:D104">
-      <x:formula1>"未確認,営業表示あり,URL・名称・運営変更,要再確認,閉鎖,除外"</x:formula1>
+      <x:formula1>"未確認,営業表示あり,URL・名称・運営変更,公式EC確認不可・閉鎖告知等,要再確認,除外"</x:formula1>
     </x:dataValidation>
     <x:dataValidation type="list" sqref="M5:M104">
       <x:formula1>"未確認,単独販売,提携店型,マーケットプレイス,不明"</x:formula1>
@@ -4533,10 +4533,10 @@
     </x:row>
     <x:row r="8" ht="32" customHeight="1">
       <x:c r="A8" s="7" t="str">
-        <x:v>確認日</x:v>
+        <x:v>現況分類日 / URL再確認日</x:v>
       </x:c>
       <x:c r="B8" s="12" t="str">
-        <x:v>2026-07-13</x:v>
+        <x:v>2026-07-13 / 2026-07-15</x:v>
       </x:c>
     </x:row>
     <x:row r="9" ht="32" customHeight="1">

</xml_diff>